<commit_message>
2D Benchmarks with Makie, some omega sweeps
</commit_message>
<xml_diff>
--- a/Results/ThesisExperimentList.xlsx
+++ b/Results/ThesisExperimentList.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\MS_BSU\SLFA_Julia\ThesisExperiments\BradenKingThesis\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A25383-BAB9-4C08-BC5E-C31844334BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B54718FE-3BA9-41B4-863B-BCE3ABB29C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" firstSheet="1" activeTab="2" xr2:uid="{C4202BFB-F5A2-4916-9270-58B282AAFCCC}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="71">
   <si>
     <t>1D Shape</t>
   </si>
@@ -257,6 +257,12 @@
   <si>
     <t>(All)</t>
   </si>
+  <si>
+    <t>ekek</t>
+  </si>
+  <si>
+    <t>oo</t>
+  </si>
 </sst>
 </file>
 
@@ -326,11 +332,63 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -387,7 +445,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -400,7 +458,11 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -409,19 +471,20 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2504,10 +2567,12 @@
   <autoFilter ref="A1:G61" xr:uid="{288A07A3-2F18-41C5-AE7D-0C571414E06A}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Composite Sine"/>
-        <filter val="Sin E"/>
-        <filter val="Sine"/>
-        <filter val="Step"/>
+        <filter val="AsymmetricRBF"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="noisy"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -4167,7 +4232,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3E51C29-A20D-4E3A-99A1-490674FEE959}">
-  <dimension ref="A1:O72"/>
+  <dimension ref="A1:O92"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -4183,1410 +4248,1410 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="20" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="18">
+      <c r="D2" s="23">
         <v>70.881799999999998</v>
       </c>
-      <c r="E2" s="19">
+      <c r="E2" s="24">
         <v>8.0158078411725396E-5</v>
       </c>
-      <c r="F2" s="19">
+      <c r="F2" s="24">
         <v>3.0149357368290598E-4</v>
       </c>
-      <c r="G2" s="19">
+      <c r="G2" s="24">
         <v>5.63382571350472E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="23" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="24">
+      <c r="D3" s="29">
         <v>16.0017</v>
       </c>
-      <c r="E3" s="25">
+      <c r="E3" s="30">
         <v>5.0852103951725701E-2</v>
       </c>
-      <c r="F3" s="25">
+      <c r="F3" s="30">
         <v>0.34232484116550099</v>
       </c>
-      <c r="G3" s="25">
+      <c r="G3" s="30">
         <v>0.67448009802876696</v>
       </c>
     </row>
     <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="26">
         <v>61.017899999999997</v>
       </c>
-      <c r="E4" s="22">
+      <c r="E4" s="27">
         <v>1.0708893831739E-4</v>
       </c>
-      <c r="F4" s="22">
+      <c r="F4" s="27">
         <v>2.5131480007299601E-4</v>
       </c>
-      <c r="G4" s="22">
+      <c r="G4" s="27">
         <v>4.22915047950317E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="20" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="26">
         <v>17.398199999999999</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="27">
         <v>0.61338183564672499</v>
       </c>
-      <c r="F5" s="22">
+      <c r="F5" s="27">
         <v>2.9628652746893702</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="27">
         <v>4.2693759980444002</v>
       </c>
     </row>
     <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="24">
+      <c r="D6" s="29">
         <v>0.272123</v>
       </c>
-      <c r="E6" s="25">
+      <c r="E6" s="30">
         <v>5.5376499405338701E-4</v>
       </c>
-      <c r="F6" s="25">
+      <c r="F6" s="30">
         <v>1.5675444224314201E-3</v>
       </c>
-      <c r="G6" s="25">
+      <c r="G6" s="30">
         <v>2.7592100881690998E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="23" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="24">
+      <c r="D7" s="29">
         <v>7.5115100000000004E-2</v>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="30">
         <v>0.23048247046100401</v>
       </c>
-      <c r="F7" s="25">
+      <c r="F7" s="30">
         <v>1.5515994839971401</v>
       </c>
-      <c r="G7" s="25">
+      <c r="G7" s="30">
         <v>2.9870621343039798</v>
       </c>
     </row>
     <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="26">
         <v>13.916399999999999</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="27">
         <v>7.4497472269780495E-5</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="27">
         <v>3.65258340649205E-4</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="27">
         <v>4.7883756930836501E-4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="20" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="26">
         <v>5.0377299999999998</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="27">
         <v>6.2147256965994498E-2</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="27">
         <v>0.75542110204059698</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="27">
         <v>1.3574724764266599</v>
       </c>
     </row>
     <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="24">
+      <c r="D10" s="29">
         <v>12.635400000000001</v>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="30">
         <v>1.82414863568795E-4</v>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="30">
         <v>9.4711775251927197E-4</v>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="30">
         <v>1.22394752256336E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="23" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="24">
+      <c r="D11" s="29">
         <v>3.9053200000000001</v>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="30">
         <v>6.6219476715996706E-2</v>
       </c>
-      <c r="F11" s="25">
+      <c r="F11" s="30">
         <v>0.41891422090307801</v>
       </c>
-      <c r="G11" s="25">
+      <c r="G11" s="30">
         <v>0.809559330529667</v>
       </c>
     </row>
     <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="21">
+      <c r="D12" s="26">
         <v>1.9495819000000001</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="27">
         <v>0.250117713343676</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="27">
         <v>1.5741567529357801</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="27">
         <v>2.8632267143095902</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="20" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="21">
+      <c r="D13" s="26">
         <v>0.54042769999999996</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="27">
         <v>0.217587732167494</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="27">
         <v>1.40379689424623</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="27">
         <v>2.72814040764188</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="23" t="s">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="24">
+      <c r="D14" s="29">
         <v>36.898899999999998</v>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="30">
         <v>2.5091416902881399E-3</v>
       </c>
-      <c r="F14" s="25">
+      <c r="F14" s="30">
         <v>7.2222514734408497E-3</v>
       </c>
-      <c r="G14" s="25">
+      <c r="G14" s="30">
         <v>1.4113510787013899E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="23" t="s">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="24">
+      <c r="D15" s="29">
         <v>7.8173300000000001</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="30">
         <v>0.801291367502725</v>
       </c>
-      <c r="F15" s="25">
+      <c r="F15" s="30">
         <v>2.88919091353198</v>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="30">
         <v>5.37246542255048</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="20" t="s">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="21">
+      <c r="D16" s="26">
         <v>47.877200000000002</v>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="27">
         <v>5.5010172994750901E-3</v>
       </c>
-      <c r="F16" s="22">
+      <c r="F16" s="27">
         <v>1.6524525225234801E-2</v>
       </c>
-      <c r="G16" s="22">
+      <c r="G16" s="27">
         <v>2.7843177139354601E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="20" t="s">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="21">
+      <c r="D17" s="26">
         <v>7.7334100000000001</v>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="27">
         <v>0.96598603616919898</v>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="27">
         <v>3.5582416127633998</v>
       </c>
-      <c r="G17" s="22">
+      <c r="G17" s="27">
         <v>6.28696568810778</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="23" t="s">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="24">
+      <c r="D18" s="29">
         <v>0.26216699999999998</v>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="30">
         <v>6.6681803044133896E-3</v>
       </c>
-      <c r="F18" s="25">
+      <c r="F18" s="30">
         <v>2.0590593675692499E-2</v>
       </c>
-      <c r="G18" s="25">
+      <c r="G18" s="30">
         <v>2.3637880091791501E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="23" t="s">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="24">
+      <c r="D19" s="29">
         <v>0.326992</v>
       </c>
-      <c r="E19" s="25">
+      <c r="E19" s="30">
         <v>2.4102050946459301</v>
       </c>
-      <c r="F19" s="25">
+      <c r="F19" s="30">
         <v>5.2920800991820203</v>
       </c>
-      <c r="G19" s="25">
+      <c r="G19" s="30">
         <v>6.77487680978372</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="20" t="s">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="21">
+      <c r="D20" s="26">
         <v>1.80654</v>
       </c>
-      <c r="E20" s="22">
+      <c r="E20" s="27">
         <v>2.6246408285867402E-3</v>
       </c>
-      <c r="F20" s="22">
+      <c r="F20" s="27">
         <v>7.3498517231258102E-3</v>
       </c>
-      <c r="G20" s="22">
+      <c r="G20" s="27">
         <v>1.4359291311023901E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="20" t="s">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="21">
+      <c r="D21" s="26">
         <v>2.6439900000000001</v>
       </c>
-      <c r="E21" s="22">
+      <c r="E21" s="27">
         <v>0.77456738695982197</v>
       </c>
-      <c r="F21" s="22">
+      <c r="F21" s="27">
         <v>2.88986608068537</v>
       </c>
-      <c r="G21" s="22">
+      <c r="G21" s="27">
         <v>5.3199692641874696</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="23" t="s">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D22" s="24">
+      <c r="D22" s="29">
         <v>2.7180300000000002</v>
       </c>
-      <c r="E22" s="25">
+      <c r="E22" s="30">
         <v>2.6246393560013302E-3</v>
       </c>
-      <c r="F22" s="25">
+      <c r="F22" s="30">
         <v>7.3498541312440697E-3</v>
       </c>
-      <c r="G22" s="25">
+      <c r="G22" s="30">
         <v>1.4359288182437299E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="23" t="s">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D23" s="24">
+      <c r="D23" s="29">
         <v>0.98388299999999995</v>
       </c>
-      <c r="E23" s="25">
+      <c r="E23" s="30">
         <v>0.65760417888491196</v>
       </c>
-      <c r="F23" s="25">
+      <c r="F23" s="30">
         <v>2.4889104970683902</v>
       </c>
-      <c r="G23" s="25">
+      <c r="G23" s="30">
         <v>4.9520824509459498</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="20" t="s">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="21">
+      <c r="D24" s="26">
         <v>4.3649449000000002</v>
       </c>
-      <c r="E24" s="22">
+      <c r="E24" s="27">
         <v>3.01868263179329E-3</v>
       </c>
-      <c r="F24" s="22">
+      <c r="F24" s="27">
         <v>9.0967723677438505E-3</v>
       </c>
-      <c r="G24" s="22">
+      <c r="G24" s="27">
         <v>1.7050883086645801E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="20" t="s">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D25" s="21">
+      <c r="D25" s="26">
         <v>2.1352106000000002</v>
       </c>
-      <c r="E25" s="22">
+      <c r="E25" s="27">
         <v>1.3240908227252699</v>
       </c>
-      <c r="F25" s="22">
+      <c r="F25" s="27">
         <v>4.4642172980045904</v>
       </c>
-      <c r="G25" s="22">
+      <c r="G25" s="27">
         <v>7.7159285101947397</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="23" t="s">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D26" s="24">
+      <c r="D26" s="29">
         <v>62.610999999999997</v>
       </c>
-      <c r="E26" s="25">
+      <c r="E26" s="30">
         <v>2.3646261766681201E-3</v>
       </c>
-      <c r="F26" s="25">
+      <c r="F26" s="30">
         <v>7.6746499836514602E-3</v>
       </c>
-      <c r="G26" s="25">
+      <c r="G26" s="30">
         <v>1.2810808666554801E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="20" t="s">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D27" s="21">
+      <c r="D27" s="26">
         <v>54.771299999999997</v>
       </c>
-      <c r="E27" s="22">
+      <c r="E27" s="27">
         <v>1.1550009147432601E-3</v>
       </c>
-      <c r="F27" s="22">
+      <c r="F27" s="27">
         <v>3.2988905937129001E-3</v>
       </c>
-      <c r="G27" s="22">
+      <c r="G27" s="27">
         <v>6.5095841618804896E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="23" t="s">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D28" s="24">
+      <c r="D28" s="29">
         <v>0.34911399999999998</v>
       </c>
-      <c r="E28" s="25">
+      <c r="E28" s="30">
         <v>6.9063927253939996E-4</v>
       </c>
-      <c r="F28" s="25">
+      <c r="F28" s="30">
         <v>2.3405484709488802E-3</v>
       </c>
-      <c r="G28" s="25">
+      <c r="G28" s="30">
         <v>3.9843163903979101E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="20" t="s">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D29" s="21">
+      <c r="D29" s="26">
         <v>2.87683</v>
       </c>
-      <c r="E29" s="22">
+      <c r="E29" s="27">
         <v>2.1818662183589101E-3</v>
       </c>
-      <c r="F29" s="22">
+      <c r="F29" s="27">
         <v>7.8308685916167308E-3</v>
       </c>
-      <c r="G29" s="22">
+      <c r="G29" s="27">
         <v>1.2375491780561699E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="23" t="s">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D30" s="24">
+      <c r="D30" s="29">
         <v>4.4576900000000004</v>
       </c>
-      <c r="E30" s="25">
+      <c r="E30" s="30">
         <v>1.9557646257379298E-3</v>
       </c>
-      <c r="F30" s="25">
+      <c r="F30" s="30">
         <v>6.7816752973434303E-3</v>
       </c>
-      <c r="G30" s="25">
+      <c r="G30" s="30">
         <v>1.12395882886645E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="20" t="s">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D31" s="21">
+      <c r="D31" s="26">
         <v>4.0496929000000002</v>
       </c>
-      <c r="E31" s="22">
+      <c r="E31" s="27">
         <v>1.93825715071022E-3</v>
       </c>
-      <c r="F31" s="22">
+      <c r="F31" s="27">
         <v>6.4403342578306603E-3</v>
       </c>
-      <c r="G31" s="22">
+      <c r="G31" s="27">
         <v>1.1390192968623499E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" s="23" t="s">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D32" s="24">
+      <c r="D32" s="29">
         <v>8.5870700000000006</v>
       </c>
-      <c r="E32" s="25">
+      <c r="E32" s="30">
         <v>4.1453415836221599E-2</v>
       </c>
-      <c r="F32" s="25">
+      <c r="F32" s="30">
         <v>0.14040456794717501</v>
       </c>
-      <c r="G32" s="25">
+      <c r="G32" s="30">
         <v>0.245064119550231</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="20" t="s">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D33" s="21">
+      <c r="D33" s="26">
         <v>14.228300000000001</v>
       </c>
-      <c r="E33" s="22">
+      <c r="E33" s="27">
         <v>0.13904915029484899</v>
       </c>
-      <c r="F33" s="22">
+      <c r="F33" s="27">
         <v>0.386911454156115</v>
       </c>
-      <c r="G33" s="22">
+      <c r="G33" s="27">
         <v>0.68318059147913801</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" s="23" t="s">
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D34" s="24">
+      <c r="D34" s="29">
         <v>7.0940500000000004E-2</v>
       </c>
-      <c r="E34" s="25">
+      <c r="E34" s="30">
         <v>0.15612056582273201</v>
       </c>
-      <c r="F34" s="25">
+      <c r="F34" s="30">
         <v>0.51286766610365897</v>
       </c>
-      <c r="G34" s="25">
+      <c r="G34" s="30">
         <v>0.71278513265916699</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" s="20" t="s">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D35" s="21">
+      <c r="D35" s="26">
         <v>1.6848399999999999</v>
       </c>
-      <c r="E35" s="22">
+      <c r="E35" s="27">
         <v>4.1456865722321698E-2</v>
       </c>
-      <c r="F35" s="22">
+      <c r="F35" s="27">
         <v>0.140393759291254</v>
       </c>
-      <c r="G35" s="22">
+      <c r="G35" s="27">
         <v>0.24506370248391099</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" s="23" t="s">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="24">
+      <c r="D36" s="29">
         <v>1.5675600000000001</v>
       </c>
-      <c r="E36" s="25">
+      <c r="E36" s="30">
         <v>4.0833320272044303E-2</v>
       </c>
-      <c r="F36" s="25">
+      <c r="F36" s="30">
         <v>0.140925650846046</v>
       </c>
-      <c r="G36" s="25">
+      <c r="G36" s="30">
         <v>0.24505734285731401</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" s="20" t="s">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D37" s="21">
+      <c r="D37" s="26">
         <v>1.2574320000000001</v>
       </c>
-      <c r="E37" s="22">
+      <c r="E37" s="27">
         <v>4.0787048159407598E-2</v>
       </c>
-      <c r="F37" s="22">
+      <c r="F37" s="27">
         <v>0.14148670760075799</v>
       </c>
-      <c r="G37" s="22">
+      <c r="G37" s="27">
         <v>0.245053054690517</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" s="23" t="s">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="B38" s="13" t="s">
+      <c r="B38" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D38" s="24">
+      <c r="D38" s="29">
         <v>54.652799999999999</v>
       </c>
-      <c r="E38" s="25">
+      <c r="E38" s="30">
         <v>4.4510542736962699E-3</v>
       </c>
-      <c r="F38" s="25">
+      <c r="F38" s="30">
         <v>1.6507426046054201E-2</v>
       </c>
-      <c r="G38" s="25">
+      <c r="G38" s="30">
         <v>2.6229440676767898E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" s="20" t="s">
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="26">
         <v>63.719700000000003</v>
       </c>
-      <c r="E39" s="22">
+      <c r="E39" s="27">
         <v>6.3331295728659403E-3</v>
       </c>
-      <c r="F39" s="22">
+      <c r="F39" s="27">
         <v>1.7931398656809299E-2</v>
       </c>
-      <c r="G39" s="22">
+      <c r="G39" s="27">
         <v>3.3279032323531001E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A40" s="23" t="s">
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="B40" s="13" t="s">
+      <c r="B40" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C40" s="13" t="s">
+      <c r="C40" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D40" s="24">
+      <c r="D40" s="29">
         <v>0.33784500000000001</v>
       </c>
-      <c r="E40" s="25">
+      <c r="E40" s="30">
         <v>1.8309538424324302E-2</v>
       </c>
-      <c r="F40" s="25">
+      <c r="F40" s="30">
         <v>8.5810910075569402E-2</v>
       </c>
-      <c r="G40" s="25">
+      <c r="G40" s="30">
         <v>8.5895394944806996E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A41" s="20" t="s">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D41" s="21">
+      <c r="D41" s="26">
         <v>2.5577700000000001</v>
       </c>
-      <c r="E41" s="22">
+      <c r="E41" s="27">
         <v>4.0142921929919003E-3</v>
       </c>
-      <c r="F41" s="22">
+      <c r="F41" s="27">
         <v>1.28594873147887E-2</v>
       </c>
-      <c r="G41" s="22">
+      <c r="G41" s="27">
         <v>2.28128592064397E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A42" s="23" t="s">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="B42" s="13" t="s">
+      <c r="B42" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C42" s="13" t="s">
+      <c r="C42" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D42" s="24">
+      <c r="D42" s="29">
         <v>3.11145</v>
       </c>
-      <c r="E42" s="25">
+      <c r="E42" s="30">
         <v>4.0142916824074297E-3</v>
       </c>
-      <c r="F42" s="25">
+      <c r="F42" s="30">
         <v>1.28594959878779E-2</v>
       </c>
-      <c r="G42" s="25">
+      <c r="G42" s="30">
         <v>2.28128717828079E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A43" s="20" t="s">
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D43" s="21">
+      <c r="D43" s="26">
         <v>4.5974335000000002</v>
       </c>
-      <c r="E43" s="22">
+      <c r="E43" s="27">
         <v>5.5891524503640499E-3</v>
       </c>
-      <c r="F43" s="22">
+      <c r="F43" s="27">
         <v>2.2443603715458799E-2</v>
       </c>
-      <c r="G43" s="22">
+      <c r="G43" s="27">
         <v>3.4773400574761498E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" s="23" t="s">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="13" t="s">
+      <c r="B44" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C44" s="13" t="s">
+      <c r="C44" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D44" s="24">
+      <c r="D44" s="29">
         <v>6.6707299999999998</v>
       </c>
-      <c r="E44" s="25">
+      <c r="E44" s="30">
         <v>0.24360513166502101</v>
       </c>
-      <c r="F44" s="25">
+      <c r="F44" s="30">
         <v>0.75915050824021502</v>
       </c>
-      <c r="G44" s="25">
+      <c r="G44" s="30">
         <v>1.51023010747413</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" s="20" t="s">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D45" s="21">
+      <c r="D45" s="26">
         <v>13.828099999999999</v>
       </c>
-      <c r="E45" s="22">
+      <c r="E45" s="27">
         <v>0.45993125581394501</v>
       </c>
-      <c r="F45" s="22">
+      <c r="F45" s="27">
         <v>1.88492546748256</v>
       </c>
-      <c r="G45" s="22">
+      <c r="G45" s="27">
         <v>3.0087160259682402</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" s="23" t="s">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="B46" s="13" t="s">
+      <c r="B46" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C46" s="13" t="s">
+      <c r="C46" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D46" s="24">
+      <c r="D46" s="29">
         <v>8.8483400000000004E-2</v>
       </c>
-      <c r="E46" s="25">
+      <c r="E46" s="30">
         <v>0.50439958268898499</v>
       </c>
-      <c r="F46" s="25">
+      <c r="F46" s="30">
         <v>1.17428808388124</v>
       </c>
-      <c r="G46" s="25">
+      <c r="G46" s="30">
         <v>1.8642873922166101</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" s="20" t="s">
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D47" s="21">
+      <c r="D47" s="26">
         <v>1.0792299999999999</v>
       </c>
-      <c r="E47" s="22">
+      <c r="E47" s="27">
         <v>0.23694535093489999</v>
       </c>
-      <c r="F47" s="22">
+      <c r="F47" s="27">
         <v>0.75638934371671995</v>
       </c>
-      <c r="G47" s="22">
+      <c r="G47" s="27">
         <v>1.51030932819276</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" s="23" t="s">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="B48" s="13" t="s">
+      <c r="B48" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C48" s="13" t="s">
+      <c r="C48" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D48" s="24">
+      <c r="D48" s="29">
         <v>1.5731599999999999</v>
       </c>
-      <c r="E48" s="25">
+      <c r="E48" s="30">
         <v>0.229718036094717</v>
       </c>
-      <c r="F48" s="25">
+      <c r="F48" s="30">
         <v>0.77961498364586002</v>
       </c>
-      <c r="G48" s="25">
+      <c r="G48" s="30">
         <v>1.4616668194278799</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A49" s="20" t="s">
+    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D49" s="21">
+      <c r="D49" s="26">
         <v>1.5713614</v>
       </c>
-      <c r="E49" s="22">
+      <c r="E49" s="27">
         <v>0.40071241252664902</v>
       </c>
-      <c r="F49" s="22">
+      <c r="F49" s="27">
         <v>0.96581405788355201</v>
       </c>
-      <c r="G49" s="22">
+      <c r="G49" s="27">
         <v>1.9214747959175</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A50" s="23" t="s">
+    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="B50" s="13" t="s">
+      <c r="B50" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C50" s="13" t="s">
+      <c r="C50" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D50" s="24">
+      <c r="D50" s="29">
         <v>6.6156800000000002</v>
       </c>
-      <c r="E50" s="25">
+      <c r="E50" s="30">
         <v>0.14592883124204001</v>
       </c>
-      <c r="F50" s="25">
+      <c r="F50" s="30">
         <v>0.60449260703643604</v>
       </c>
-      <c r="G50" s="25">
+      <c r="G50" s="30">
         <v>1.0055006730877001</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A51" s="20" t="s">
+    <row r="51" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D51" s="21">
+      <c r="D51" s="26">
         <v>35.988700000000001</v>
       </c>
-      <c r="E51" s="22">
+      <c r="E51" s="27">
         <v>0.12968113651434601</v>
       </c>
-      <c r="F51" s="22">
+      <c r="F51" s="27">
         <v>0.57749149831848201</v>
       </c>
-      <c r="G51" s="22">
+      <c r="G51" s="27">
         <v>1.0185314034547699</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A52" s="23" t="s">
+    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="B52" s="13" t="s">
+      <c r="B52" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C52" s="13" t="s">
+      <c r="C52" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D52" s="24">
+      <c r="D52" s="29">
         <v>0.292354</v>
       </c>
-      <c r="E52" s="25">
+      <c r="E52" s="30">
         <v>0.31220361801305802</v>
       </c>
-      <c r="F52" s="25">
+      <c r="F52" s="30">
         <v>0.73540788758055997</v>
       </c>
-      <c r="G52" s="25">
+      <c r="G52" s="30">
         <v>0.73616458940486895</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A53" s="20" t="s">
+    <row r="53" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="B53" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C53" s="6" t="s">
+      <c r="C53" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D53" s="21">
+      <c r="D53" s="26">
         <v>13.1905</v>
       </c>
-      <c r="E53" s="22">
+      <c r="E53" s="27">
         <v>3.3790369124594198E-3</v>
       </c>
-      <c r="F53" s="22">
+      <c r="F53" s="27">
         <v>1.0685154303572E-2</v>
       </c>
-      <c r="G53" s="22">
+      <c r="G53" s="27">
         <v>1.9292474326642099E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A54" s="23" t="s">
+    <row r="54" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="B54" s="13" t="s">
+      <c r="B54" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C54" s="13" t="s">
+      <c r="C54" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D54" s="24">
+      <c r="D54" s="29">
         <v>1.1140000000000001</v>
       </c>
-      <c r="E54" s="25">
+      <c r="E54" s="30">
         <v>0.249127964789603</v>
       </c>
-      <c r="F54" s="25">
+      <c r="F54" s="30">
         <v>0.88938504322949796</v>
       </c>
-      <c r="G54" s="25">
+      <c r="G54" s="30">
         <v>1.3298393318872299</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A55" s="20" t="s">
+    <row r="55" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="B55" s="6" t="s">
+      <c r="B55" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="C55" s="6" t="s">
+      <c r="C55" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D55" s="21">
+      <c r="D55" s="26">
         <v>1.9451883000000001</v>
       </c>
-      <c r="E55" s="22">
+      <c r="E55" s="27">
         <v>0.40359911336578402</v>
       </c>
-      <c r="F55" s="22">
+      <c r="F55" s="27">
         <v>0.62498700848665001</v>
       </c>
-      <c r="G55" s="22">
+      <c r="G55" s="27">
         <v>1.1677899083337999</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A56" s="23" t="s">
+    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="B56" s="13" t="s">
+      <c r="B56" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C56" s="13" t="s">
+      <c r="C56" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D56" s="24">
+      <c r="D56" s="29">
         <v>9.6140600000000003</v>
       </c>
-      <c r="E56" s="25">
+      <c r="E56" s="30">
         <v>9.8471561707902805E-2</v>
       </c>
-      <c r="F56" s="25">
+      <c r="F56" s="30">
         <v>0.33753961371707603</v>
       </c>
-      <c r="G56" s="25">
+      <c r="G56" s="30">
         <v>0.61523698654407699</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A57" s="20" t="s">
+    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="B57" s="6" t="s">
+      <c r="B57" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C57" s="6" t="s">
+      <c r="C57" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D57" s="21">
+      <c r="D57" s="26">
         <v>17.239699999999999</v>
       </c>
-      <c r="E57" s="22">
+      <c r="E57" s="27">
         <v>0.14224438082638899</v>
       </c>
-      <c r="F57" s="22">
+      <c r="F57" s="27">
         <v>0.414745195132116</v>
       </c>
-      <c r="G57" s="22">
+      <c r="G57" s="27">
         <v>0.80134390579414105</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A58" s="23" t="s">
+    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A58" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="B58" s="13" t="s">
+      <c r="B58" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C58" s="13" t="s">
+      <c r="C58" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D58" s="24">
+      <c r="D58" s="29">
         <v>6.8042199999999997E-2</v>
       </c>
-      <c r="E58" s="25">
+      <c r="E58" s="30">
         <v>0.50760907712574199</v>
       </c>
-      <c r="F58" s="25">
+      <c r="F58" s="30">
         <v>1.09124651945925</v>
       </c>
-      <c r="G58" s="25">
+      <c r="G58" s="30">
         <v>1.10549516064681</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A59" s="20" t="s">
+    <row r="59" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="B59" s="6" t="s">
+      <c r="B59" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D59" s="21">
+      <c r="D59" s="26">
         <v>3.1019899999999998</v>
       </c>
-      <c r="E59" s="22">
+      <c r="E59" s="27">
         <v>9.8036203584847603E-2</v>
       </c>
-      <c r="F59" s="22">
+      <c r="F59" s="27">
         <v>0.30778567176863803</v>
       </c>
-      <c r="G59" s="22">
+      <c r="G59" s="27">
         <v>0.58570046607555803</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A60" s="23" t="s">
+    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="B60" s="13" t="s">
+      <c r="B60" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C60" s="13" t="s">
+      <c r="C60" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D60" s="24">
+      <c r="D60" s="29">
         <v>2.7850799999999998</v>
       </c>
-      <c r="E60" s="25">
+      <c r="E60" s="30">
         <v>9.71806155299062E-2</v>
       </c>
-      <c r="F60" s="25">
+      <c r="F60" s="30">
         <v>0.295448031130705</v>
       </c>
-      <c r="G60" s="25">
+      <c r="G60" s="30">
         <v>0.57115690156416798</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A61" s="20" t="s">
+    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="B61" s="6" t="s">
+      <c r="B61" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="C61" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D61" s="21">
+      <c r="D61" s="26">
         <v>0.69017720000000005</v>
       </c>
-      <c r="E61" s="22">
+      <c r="E61" s="27">
         <v>0.131432654739953</v>
       </c>
-      <c r="F61" s="22">
+      <c r="F61" s="27">
         <v>0.54299357139798299</v>
       </c>
-      <c r="G61" s="22">
+      <c r="G61" s="27">
         <v>1.0098621954920799</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="K62" s="7" t="s">
+      <c r="K62" s="11" t="s">
         <v>37</v>
       </c>
       <c r="L62" t="s">
@@ -5594,7 +5659,7 @@
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="K63" s="7" t="s">
+      <c r="K63" s="11" t="s">
         <v>36</v>
       </c>
       <c r="L63" t="s">
@@ -5602,7 +5667,7 @@
       </c>
     </row>
     <row r="65" spans="11:15" x14ac:dyDescent="0.35">
-      <c r="K65" s="7" t="s">
+      <c r="K65" s="11" t="s">
         <v>55</v>
       </c>
       <c r="L65" t="s">
@@ -5619,122 +5684,180 @@
       </c>
     </row>
     <row r="66" spans="11:15" x14ac:dyDescent="0.35">
-      <c r="K66" s="8" t="s">
+      <c r="K66" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="L66" s="11">
+      <c r="L66" s="15">
         <v>28.035107</v>
       </c>
-      <c r="M66" s="12">
+      <c r="M66" s="16">
         <v>0.13910073921247004</v>
       </c>
-      <c r="N66" s="12">
+      <c r="N66" s="16">
         <v>0.51048088727152119</v>
       </c>
-      <c r="O66" s="12">
+      <c r="O66" s="16">
         <v>0.94766945499370725</v>
       </c>
     </row>
     <row r="67" spans="11:15" x14ac:dyDescent="0.35">
-      <c r="K67" s="8" t="s">
+      <c r="K67" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="L67" s="11">
+      <c r="L67" s="15">
         <v>33.380251000000001</v>
       </c>
-      <c r="M67" s="12">
+      <c r="M67" s="16">
         <v>0.24633700319908547</v>
       </c>
-      <c r="N67" s="12">
+      <c r="N67" s="16">
         <v>0.98231866318178729</v>
       </c>
-      <c r="O67" s="12">
+      <c r="O67" s="16">
         <v>1.6136168321521187</v>
       </c>
     </row>
     <row r="68" spans="11:15" x14ac:dyDescent="0.35">
-      <c r="K68" s="8" t="s">
+      <c r="K68" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="L68" s="11">
+      <c r="L68" s="15">
         <v>0.21431762000000001</v>
       </c>
-      <c r="M68" s="12">
+      <c r="M68" s="16">
         <v>0.41472425317527806</v>
       </c>
-      <c r="N68" s="12">
+      <c r="N68" s="16">
         <v>1.0467799336848513</v>
       </c>
-      <c r="O68" s="12">
+      <c r="O68" s="16">
         <v>1.429694802053032</v>
       </c>
     </row>
     <row r="69" spans="11:15" x14ac:dyDescent="0.35">
-      <c r="K69" s="8" t="s">
+      <c r="K69" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="L69" s="11">
+      <c r="L69" s="15">
         <v>4.7895820000000002</v>
       </c>
-      <c r="M69" s="12">
+      <c r="M69" s="16">
         <v>0.12254273977925523</v>
       </c>
-      <c r="N69" s="12">
+      <c r="N69" s="16">
         <v>0.48889465777763313</v>
       </c>
-      <c r="O69" s="12">
+      <c r="O69" s="16">
         <v>0.90878341915603333</v>
       </c>
     </row>
     <row r="70" spans="11:15" x14ac:dyDescent="0.35">
-      <c r="K70" s="8" t="s">
+      <c r="K70" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="L70" s="11">
+      <c r="L70" s="15">
         <v>3.4851573</v>
       </c>
-      <c r="M70" s="12">
+      <c r="M70" s="16">
         <v>0.13494607028148947</v>
       </c>
-      <c r="N70" s="12">
+      <c r="N70" s="16">
         <v>0.50411365699925614</v>
       </c>
-      <c r="O70" s="12">
+      <c r="O70" s="16">
         <v>0.94189978729886814</v>
       </c>
     </row>
     <row r="71" spans="11:15" x14ac:dyDescent="0.35">
-      <c r="K71" s="8" t="s">
+      <c r="K71" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="L71" s="11">
+      <c r="L71" s="15">
         <v>2.3101450400000005</v>
       </c>
-      <c r="M71" s="12">
+      <c r="M71" s="16">
         <v>0.27788735892611011</v>
       </c>
-      <c r="N71" s="12">
+      <c r="N71" s="16">
         <v>0.97554330008965773</v>
       </c>
-      <c r="O71" s="12">
+      <c r="O71" s="16">
         <v>1.7714690063210139</v>
       </c>
     </row>
     <row r="72" spans="11:15" x14ac:dyDescent="0.35">
-      <c r="K72" s="8" t="s">
+      <c r="K72" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="L72" s="11">
+      <c r="L72" s="15">
         <v>12.035759993333333</v>
       </c>
-      <c r="M72" s="10">
+      <c r="M72" s="14">
         <v>0.22258969409561474</v>
       </c>
-      <c r="N72" s="10">
+      <c r="N72" s="14">
         <v>0.75135518316745076</v>
       </c>
-      <c r="O72" s="10">
+      <c r="O72" s="14">
         <v>1.268855550329129</v>
+      </c>
+    </row>
+    <row r="79" spans="11:15" x14ac:dyDescent="0.35">
+      <c r="M79" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="80" spans="11:15" x14ac:dyDescent="0.35">
+      <c r="M80" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="81" spans="11:14" x14ac:dyDescent="0.35">
+      <c r="M81" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="82" spans="11:14" x14ac:dyDescent="0.35">
+      <c r="M82" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="N82" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="83" spans="11:14" x14ac:dyDescent="0.35">
+      <c r="M83" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="84" spans="11:14" x14ac:dyDescent="0.35">
+      <c r="M84" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="88" spans="11:14" x14ac:dyDescent="0.35">
+      <c r="K88" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="89" spans="11:14" x14ac:dyDescent="0.35">
+      <c r="K89" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="90" spans="11:14" x14ac:dyDescent="0.35">
+      <c r="K90" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="91" spans="11:14" x14ac:dyDescent="0.35">
+      <c r="K91" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="92" spans="11:14" x14ac:dyDescent="0.35">
+      <c r="K92" s="18" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -5755,7 +5878,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="11" t="s">
         <v>55</v>
       </c>
       <c r="B3" t="s">
@@ -5763,50 +5886,50 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="13">
         <v>29.022560999999996</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="13">
         <v>32.52543099999999</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="13">
         <v>0.21369023000000001</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="13">
         <v>4.8820490000000003</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="13">
         <v>3.6192212999999995</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="13">
         <v>14.052590505999996</v>
       </c>
     </row>
@@ -5825,7 +5948,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="11" t="s">
         <v>55</v>
       </c>
       <c r="B1" t="s">
@@ -5833,50 +5956,50 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="13">
         <v>20.114168810000002</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="13">
         <v>10.906844200000002</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="13">
         <v>15.12046445</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="13">
         <v>15.12046445</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="13">
         <v>9.0010106199999989</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="13">
         <v>14.052590506000001</v>
       </c>
     </row>
@@ -6944,7 +7067,7 @@
       <c r="C53" t="s">
         <v>64</v>
       </c>
-      <c r="D53" s="10">
+      <c r="D53" s="14">
         <v>7.4497472269780495E-5</v>
       </c>
       <c r="E53">
@@ -6964,7 +7087,7 @@
       <c r="C54" t="s">
         <v>64</v>
       </c>
-      <c r="D54" s="10">
+      <c r="D54" s="14">
         <v>8.0158078411725396E-5</v>
       </c>
       <c r="E54">

</xml_diff>